<commit_message>
Fix v1 summaries and LAND basis flagged in issue #1
- STEPI 367: describe the 53 firms as companies with a past valuation of 1 trillion won or more
- 혁신의숲: drop paywalled figures, note the members-only status in 비고
- Report: add the 연구성과 이관·추적관리 detail to the LAND description

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/이전버전/결과/딥테크_정책동향_2026-10-17.xlsx
+++ b/이전버전/결과/딥테크_정책동향_2026-10-17.xlsx
@@ -282,7 +282,7 @@
     <t>STEPI Insight 제367호 「국내외 유니콘 현황과 정책 과제」</t>
   </si>
   <si>
-    <t>국내 유니콘 53개사를 실질 독립성과 벤처투자 기반 성장 여부로 다시 분류한 결과, 실질 유니콘은 35개사로 나타났다. Series A에서 B로 넘어가는 단계가 가장 큰 병목이고, 설립 후 6~8년 구간이 지원 공백으로 확인됐다. 유니콘 수를 단순히 늘리는 목표 대신 전환율과 딥테크 비중 같은 복합 성과지표로 관리할 것을 제안했다.</t>
+    <t xml:space="preserve">기업가치 1조 원 이상 이력이 있는 국내 기업 53개사를 실질 독립성과 벤처투자 기반 성장 여부로 재분류해 실질 유니콘 35개사(유니콘 22·엑싯콘 9·유니콥스 2·좀비콘 2)를 도출했다. Series A에서 B로 넘어가는 단계가 가장 큰 병목이고, 설립 후 6~8년 구간이 지원 공백으로 확인됐다. 유니콘 수 대신 단계 전환율과 딥테크 비중 같은 복합 성과지표로 관리할 것을 제안했다.</t>
   </si>
   <si>
     <t>저자: 김선우, 이윤아</t>
@@ -609,10 +609,10 @@
     <t>2026년 7월 스타트업 투자결산: 로보틱스가 판을 바꿨다…제조/하드웨어 투자금액 1위</t>
   </si>
   <si>
-    <t>2026년 7월 신규 투자를 받은 스타트업은 140개사, 투자금은 9,821억원으로 6월보다 금액 39.5%, 건수 21.7% 늘었다. AI·딥테크·블록체인 분야가 40건(28.6%)으로 건수 1위, 금액은 2,567억원(26.1%)으로 2위였다. 제조·하드웨어 분야가 3,146억원(32.0%)으로 처음 금액 1위에 올랐다.</t>
-  </si>
-  <si>
-    <t>민간 투자 데이터 플랫폼 집계(정부 승인통계 아님) / 통합 검증: 제목은 확인, 본문 수치는 텍스트로 대조 불가(보고서에는 수치 미사용)</t>
+    <t xml:space="preserve">2026년 7월 스타트업 투자 결산. 제목 기준으로 로보틱스를 중심으로 제조·하드웨어 분야가 투자금액 1위를 기록함. 본문 수치는 유료 회원 전용이라 싣지 않음.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">민간 투자 데이터 플랫폼 집계(정부 승인통계 아님) / 통합 검증: 제목은 확인, 본문 수치는 텍스트로 대조 불가(보고서에는 수치 미사용) / 유료 회원 전용 글(isAccessibleForFree: false): 공개된 제목 범위만 사용</t>
   </si>
   <si>
     <t>https://www.oecd.org/en/publications/what-it-takes-for-start-ups-to-scale-up_1f743fa7-en.html</t>

</xml_diff>